<commit_message>
App created and deployed on AWS
</commit_message>
<xml_diff>
--- a/outputs/optuna/performance_over_baseline.xlsx
+++ b/outputs/optuna/performance_over_baseline.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kushagra Saxena\Documents\enam-skills-assessment\outputs\optuna\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{60C8A818-A180-46AC-AB92-5383A19F8CE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{692FF0B7-80FE-4099-86CF-DEA46C30EDB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="22620" windowHeight="13500" xr2:uid="{87A4CA6C-0E8C-487D-9B00-BDFE252D82DD}"/>
+    <workbookView xWindow="4650" yWindow="2760" windowWidth="16800" windowHeight="9680" xr2:uid="{87A4CA6C-0E8C-487D-9B00-BDFE252D82DD}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -493,7 +493,6 @@
     <col min="3" max="3" width="10.90625" customWidth="1"/>
     <col min="4" max="4" width="11.54296875" customWidth="1"/>
     <col min="5" max="5" width="23.81640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:5" x14ac:dyDescent="0.35">
@@ -518,7 +517,7 @@
         <v>0.33</v>
       </c>
       <c r="D3" s="1">
-        <v>0.89949999999999997</v>
+        <v>0.899752</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>11</v>
@@ -532,7 +531,7 @@
         <v>0.01</v>
       </c>
       <c r="D4" s="1">
-        <v>3.78E-2</v>
+        <v>3.7807E-2</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>12</v>
@@ -546,7 +545,7 @@
         <v>1</v>
       </c>
       <c r="D5" s="1">
-        <v>2.37</v>
+        <v>2.374657</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>24</v>
@@ -560,7 +559,7 @@
         <v>0.02</v>
       </c>
       <c r="D6" s="1">
-        <v>0.11849999999999999</v>
+        <v>0.11815299999999999</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>23</v>
@@ -574,7 +573,7 @@
         <v>1.1499999999999999</v>
       </c>
       <c r="D7" s="1">
-        <v>1.22</v>
+        <v>1.220966</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>13</v>
@@ -588,7 +587,7 @@
         <v>50</v>
       </c>
       <c r="D8" s="1">
-        <v>44.5</v>
+        <v>44.494370000000004</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>14</v>
@@ -602,7 +601,7 @@
         <v>0.4</v>
       </c>
       <c r="D9" s="1">
-        <v>0.28689999999999999</v>
+        <v>0.28690300000000002</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>15</v>

</xml_diff>